<commit_message>
Fixed R4 -> 510ohm
</commit_message>
<xml_diff>
--- a/hardware/board/harp.peripheral.poke-port/fab_files/BOM harp.peripheral.poke-port.xlsx
+++ b/hardware/board/harp.peripheral.poke-port/fab_files/BOM harp.peripheral.poke-port.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nathan/Documents/Work/Git/harp.peripheral.poke-port/hardware/board/harp.peripheral.poke-port/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nathan/Documents/Work/Git/harp.peripheral.poke-port/hardware/board/harp.peripheral.poke-port/fab_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60CB0D37-2970-A540-9400-2A1D77CC4023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86AC85E2-F286-8447-8D7B-3831ED744325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="300" yWindow="740" windowWidth="22340" windowHeight="17360" xr2:uid="{E49442E1-C0EC-3F4B-978D-06B74820C73C}"/>
+    <workbookView xWindow="15300" yWindow="1600" windowWidth="22340" windowHeight="17360" xr2:uid="{E49442E1-C0EC-3F4B-978D-06B74820C73C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="91">
   <si>
     <t>Designator</t>
   </si>
@@ -74,9 +74,6 @@
     <t>TPS63060</t>
   </si>
   <si>
-    <t>R1,R2,R4</t>
-  </si>
-  <si>
     <t>R_0603_1608Metric</t>
   </si>
   <si>
@@ -297,6 +294,21 @@
   </si>
   <si>
     <t>QTY</t>
+  </si>
+  <si>
+    <t>R1,R2</t>
+  </si>
+  <si>
+    <t>R4</t>
+  </si>
+  <si>
+    <t>2019-SG73P1JTTD5100FCT-ND</t>
+  </si>
+  <si>
+    <t>SG73P1JTTD5100F</t>
+  </si>
+  <si>
+    <t>RES 510 OHM 1% 1/3W 0603</t>
   </si>
 </sst>
 </file>
@@ -683,7 +695,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0557E55-AD76-C246-823D-29035C04EC52}">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="4" width="17" customWidth="1"/>
@@ -698,22 +710,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>37</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>2</v>
@@ -724,16 +736,16 @@
         <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>60</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>4</v>
@@ -750,16 +762,16 @@
         <v>6</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>70</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>7</v>
@@ -776,16 +788,16 @@
         <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>10</v>
@@ -799,25 +811,25 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C5" t="s">
-        <v>73</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="G5" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H5" s="2">
         <v>100</v>
@@ -825,236 +837,262 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>14</v>
+        <v>87</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>76</v>
+        <v>88</v>
+      </c>
+      <c r="C6" t="s">
+        <v>89</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G6" s="2">
         <v>1</v>
       </c>
       <c r="H6" s="2">
-        <v>127</v>
+        <v>510</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G7" s="2">
         <v>1</v>
       </c>
-      <c r="H7" s="2" t="s">
-        <v>17</v>
+      <c r="H7" s="2">
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>64</v>
+        <v>81</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="G8" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="G9" s="2">
         <v>2</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="G10" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>83</v>
+        <v>53</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>84</v>
+        <v>52</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>85</v>
+        <v>54</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="G11" s="2">
         <v>1</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>50</v>
+        <v>82</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>30</v>
+        <v>83</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>51</v>
+        <v>84</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="G12" s="2">
         <v>1</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="G13" s="2">
         <v>1</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G14" s="2">
         <v>1</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G15" s="2">
+        <v>1</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>